<commit_message>
v1.2.0: demo B2 blank + byte-exact demo files; version single source in UI; trace guide S2 template; screenshot fixes; release docs
</commit_message>
<xml_diff>
--- a/demo/mc_v12/site_A/02_MCDEMO-A_课题二重构指标_模拟数据_仅供测试演示.xlsx
+++ b/demo/mc_v12/site_A/02_MCDEMO-A_课题二重构指标_模拟数据_仅供测试演示.xlsx
@@ -544,14 +544,10 @@
           <t>场地编号</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>MCDEMO-A</t>
-        </is>
-      </c>
+      <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>必填, 与系统中场地编号一致</t>
+          <t>可留空(以页面所选场地为准); 填写时须与系统中场地编号一致</t>
         </is>
       </c>
     </row>

</xml_diff>